<commit_message>
pricing quote button text
</commit_message>
<xml_diff>
--- a/ClearSiteCo_Client_Content_Review (1).xlsx
+++ b/ClearSiteCo_Client_Content_Review (1).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11580"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Editable Content" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2314" uniqueCount="674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2314" uniqueCount="673">
   <si>
     <t>Section Order</t>
   </si>
@@ -1380,29 +1380,6 @@
     <t>Reliable communication and great attention to common areas. They make handovers and recurring strata cleans much easier to manage.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Will provide you with 5 client reviews via email.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
     <t>testimonials.2.rating</t>
   </si>
   <si>
@@ -2129,7 +2106,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2149,13 +2126,6 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2311,7 +2281,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2345,12 +2315,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEAF5FF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2677,10 +2641,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2689,37 +2656,37 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2734,77 +2701,74 @@
     <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2835,31 +2799,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7901,7 +7859,7 @@
         <v>434</v>
       </c>
       <c r="H115" s="13" t="s">
-        <v>435</v>
+        <v>415</v>
       </c>
       <c r="I115" s="8" t="s">
         <v>20</v>
@@ -7933,7 +7891,7 @@
         <v>404</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>417</v>
@@ -7951,7 +7909,7 @@
         <v>57</v>
       </c>
       <c r="K116" s="6" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L116" s="6" t="s">
         <v>23</v>
@@ -7965,39 +7923,39 @@
         <v>13</v>
       </c>
       <c r="B117" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="C117" s="16" t="s">
         <v>438</v>
       </c>
-      <c r="C117" s="16" t="s">
+      <c r="D117" s="16" t="s">
         <v>439</v>
       </c>
-      <c r="D117" s="16" t="s">
+      <c r="E117" s="16" t="s">
         <v>440</v>
-      </c>
-      <c r="E117" s="16" t="s">
-        <v>441</v>
       </c>
       <c r="F117" s="16" t="s">
         <v>152</v>
       </c>
       <c r="G117" s="16" t="s">
+        <v>441</v>
+      </c>
+      <c r="H117" s="17" t="s">
         <v>442</v>
       </c>
-      <c r="H117" s="17" t="s">
-        <v>443</v>
-      </c>
       <c r="I117" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="J117" s="18" t="s">
-        <v>348</v>
-      </c>
-      <c r="K117" s="19" t="s">
-        <v>437</v>
-      </c>
-      <c r="L117" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="M117" s="19" t="s">
+      <c r="J117" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K117" s="16" t="s">
+        <v>436</v>
+      </c>
+      <c r="L117" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M117" s="16" t="s">
         <v>24</v>
       </c>
     </row>
@@ -8006,34 +7964,34 @@
         <v>13</v>
       </c>
       <c r="B118" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C118" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="C118" s="2" t="s">
+      <c r="D118" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="D118" s="2" t="s">
-        <v>440</v>
-      </c>
       <c r="E118" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F118" s="2" t="s">
         <v>156</v>
       </c>
       <c r="G118" s="12" t="s">
+        <v>444</v>
+      </c>
+      <c r="H118" s="13" t="s">
         <v>445</v>
       </c>
-      <c r="H118" s="13" t="s">
+      <c r="I118" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J118" s="14" t="s">
         <v>446</v>
       </c>
-      <c r="I118" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J118" s="14" t="s">
-        <v>447</v>
-      </c>
       <c r="K118" s="6" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L118" s="6" t="s">
         <v>23</v>
@@ -8047,34 +8005,34 @@
         <v>13</v>
       </c>
       <c r="B119" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="C119" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="C119" s="6" t="s">
+      <c r="D119" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="D119" s="6" t="s">
-        <v>440</v>
-      </c>
       <c r="E119" s="6" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F119" s="6" t="s">
         <v>161</v>
       </c>
       <c r="G119" s="14" t="s">
+        <v>448</v>
+      </c>
+      <c r="H119" s="13" t="s">
         <v>449</v>
       </c>
-      <c r="H119" s="13" t="s">
+      <c r="I119" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J119" s="12" t="s">
         <v>450</v>
       </c>
-      <c r="I119" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J119" s="12" t="s">
-        <v>451</v>
-      </c>
       <c r="K119" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L119" s="2" t="s">
         <v>23</v>
@@ -8088,22 +8046,22 @@
         <v>13</v>
       </c>
       <c r="B120" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C120" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="C120" s="2" t="s">
+      <c r="D120" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="D120" s="2" t="s">
-        <v>440</v>
-      </c>
       <c r="E120" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="F120" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="F120" s="2" t="s">
+      <c r="G120" s="12" t="s">
         <v>453</v>
-      </c>
-      <c r="G120" s="12" t="s">
-        <v>454</v>
       </c>
       <c r="H120" s="7"/>
       <c r="I120" s="8" t="s">
@@ -8113,7 +8071,7 @@
         <v>57</v>
       </c>
       <c r="K120" s="6" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L120" s="6" t="s">
         <v>23</v>
@@ -8127,23 +8085,23 @@
         <v>13</v>
       </c>
       <c r="B121" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="C121" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="C121" s="6" t="s">
+      <c r="D121" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="D121" s="6" t="s">
-        <v>440</v>
-      </c>
       <c r="E121" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="F121" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="G121" s="14" t="s">
         <v>455</v>
       </c>
-      <c r="F121" s="6" t="s">
-        <v>453</v>
-      </c>
-      <c r="G121" s="14" t="s">
-        <v>456</v>
-      </c>
       <c r="H121" s="7" t="s">
         <v>57</v>
       </c>
@@ -8154,7 +8112,7 @@
         <v>57</v>
       </c>
       <c r="K121" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L121" s="2" t="s">
         <v>23</v>
@@ -8168,34 +8126,34 @@
         <v>13</v>
       </c>
       <c r="B122" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C122" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="C122" s="2" t="s">
+      <c r="D122" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="D122" s="2" t="s">
-        <v>440</v>
-      </c>
       <c r="E122" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="G122" s="12" t="s">
         <v>457</v>
       </c>
-      <c r="F122" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="G122" s="12" t="s">
+      <c r="H122" s="13" t="s">
         <v>458</v>
       </c>
-      <c r="H122" s="13" t="s">
-        <v>459</v>
-      </c>
       <c r="I122" s="8" t="s">
         <v>20</v>
       </c>
       <c r="J122" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="K122" s="6" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L122" s="6" t="s">
         <v>23</v>
@@ -8209,25 +8167,25 @@
         <v>13</v>
       </c>
       <c r="B123" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="C123" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="C123" s="6" t="s">
+      <c r="D123" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="D123" s="6" t="s">
-        <v>440</v>
-      </c>
       <c r="E123" s="6" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F123" s="6" t="s">
         <v>183</v>
       </c>
       <c r="G123" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="H123" s="13" t="s">
         <v>461</v>
-      </c>
-      <c r="H123" s="13" t="s">
-        <v>462</v>
       </c>
       <c r="I123" s="8" t="s">
         <v>20</v>
@@ -8236,7 +8194,7 @@
         <v>38</v>
       </c>
       <c r="K123" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L123" s="2" t="s">
         <v>23</v>
@@ -8250,34 +8208,34 @@
         <v>13</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C124" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D124" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D124" s="2" t="s">
+      <c r="E124" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="E124" s="2" t="s">
+      <c r="F124" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="F124" s="2" t="s">
+      <c r="G124" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="G124" s="2" t="s">
+      <c r="H124" s="13" t="s">
         <v>467</v>
       </c>
-      <c r="H124" s="13" t="s">
-        <v>468</v>
-      </c>
       <c r="I124" s="8" t="s">
         <v>20</v>
       </c>
       <c r="J124" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="K124" s="6" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L124" s="6" t="s">
         <v>23</v>
@@ -8291,23 +8249,23 @@
         <v>13</v>
       </c>
       <c r="B125" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C125" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="D125" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="D125" s="6" t="s">
-        <v>464</v>
-      </c>
       <c r="E125" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="F125" s="6" t="s">
         <v>469</v>
       </c>
-      <c r="F125" s="6" t="s">
+      <c r="G125" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="G125" s="6" t="s">
-        <v>471</v>
-      </c>
       <c r="H125" s="7" t="s">
         <v>57</v>
       </c>
@@ -8318,7 +8276,7 @@
         <v>57</v>
       </c>
       <c r="K125" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L125" s="2" t="s">
         <v>23</v>
@@ -8332,23 +8290,23 @@
         <v>13</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C126" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D126" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D126" s="2" t="s">
-        <v>464</v>
-      </c>
       <c r="E126" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="F126" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="F126" s="2" t="s">
+      <c r="G126" s="12" t="s">
         <v>473</v>
       </c>
-      <c r="G126" s="12" t="s">
-        <v>474</v>
-      </c>
       <c r="H126" s="7" t="s">
         <v>57</v>
       </c>
@@ -8359,7 +8317,7 @@
         <v>57</v>
       </c>
       <c r="K126" s="6" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L126" s="6" t="s">
         <v>23</v>
@@ -8373,34 +8331,34 @@
         <v>13</v>
       </c>
       <c r="B127" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C127" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="D127" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="D127" s="6" t="s">
-        <v>464</v>
-      </c>
       <c r="E127" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="F127" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="F127" s="6" t="s">
+      <c r="G127" s="14" t="s">
         <v>476</v>
       </c>
-      <c r="G127" s="14" t="s">
+      <c r="H127" s="13" t="s">
         <v>477</v>
       </c>
-      <c r="H127" s="13" t="s">
-        <v>478</v>
-      </c>
       <c r="I127" s="8" t="s">
         <v>20</v>
       </c>
       <c r="J127" s="12" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="K127" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="L127" s="2" t="s">
         <v>23</v>
@@ -8414,25 +8372,25 @@
         <v>13</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C128" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D128" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D128" s="2" t="s">
-        <v>464</v>
-      </c>
       <c r="E128" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="F128" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="F128" s="2" t="s">
+      <c r="G128" s="12" t="s">
         <v>480</v>
       </c>
-      <c r="G128" s="12" t="s">
+      <c r="H128" s="13" t="s">
         <v>481</v>
-      </c>
-      <c r="H128" s="13" t="s">
-        <v>482</v>
       </c>
       <c r="I128" s="8" t="s">
         <v>20</v>
@@ -8441,10 +8399,10 @@
         <v>348</v>
       </c>
       <c r="K128" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="L128" s="6" t="s">
         <v>483</v>
-      </c>
-      <c r="L128" s="6" t="s">
-        <v>484</v>
       </c>
       <c r="M128" s="6" t="s">
         <v>24</v>
@@ -8455,25 +8413,25 @@
         <v>13</v>
       </c>
       <c r="B129" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C129" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="D129" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="D129" s="6" t="s">
-        <v>464</v>
-      </c>
       <c r="E129" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="F129" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="G129" s="6" t="s">
         <v>485</v>
       </c>
-      <c r="F129" s="6" t="s">
-        <v>466</v>
-      </c>
-      <c r="G129" s="6" t="s">
+      <c r="H129" s="13" t="s">
         <v>486</v>
-      </c>
-      <c r="H129" s="13" t="s">
-        <v>487</v>
       </c>
       <c r="I129" s="8" t="s">
         <v>20</v>
@@ -8482,10 +8440,10 @@
         <v>38</v>
       </c>
       <c r="K129" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="L129" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="L129" s="2" t="s">
-        <v>484</v>
       </c>
       <c r="M129" s="2" t="s">
         <v>24</v>
@@ -8496,25 +8454,25 @@
         <v>13</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C130" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D130" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D130" s="2" t="s">
-        <v>464</v>
-      </c>
       <c r="E130" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="G130" s="2" t="s">
         <v>488</v>
       </c>
-      <c r="F130" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="G130" s="2" t="s">
+      <c r="H130" s="13" t="s">
         <v>489</v>
-      </c>
-      <c r="H130" s="13" t="s">
-        <v>490</v>
       </c>
       <c r="I130" s="8" t="s">
         <v>20</v>
@@ -8523,10 +8481,10 @@
         <v>348</v>
       </c>
       <c r="K130" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="L130" s="6" t="s">
         <v>483</v>
-      </c>
-      <c r="L130" s="6" t="s">
-        <v>484</v>
       </c>
       <c r="M130" s="6" t="s">
         <v>24</v>
@@ -8537,25 +8495,25 @@
         <v>13</v>
       </c>
       <c r="B131" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C131" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="D131" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="D131" s="6" t="s">
-        <v>464</v>
-      </c>
       <c r="E131" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="F131" s="6" t="s">
+        <v>472</v>
+      </c>
+      <c r="G131" s="6" t="s">
         <v>491</v>
       </c>
-      <c r="F131" s="6" t="s">
-        <v>473</v>
-      </c>
-      <c r="G131" s="6" t="s">
+      <c r="H131" s="13" t="s">
         <v>492</v>
-      </c>
-      <c r="H131" s="13" t="s">
-        <v>493</v>
       </c>
       <c r="I131" s="8" t="s">
         <v>20</v>
@@ -8564,10 +8522,10 @@
         <v>348</v>
       </c>
       <c r="K131" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="L131" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="L131" s="2" t="s">
-        <v>484</v>
       </c>
       <c r="M131" s="2" t="s">
         <v>24</v>
@@ -8578,25 +8536,25 @@
         <v>13</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C132" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D132" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D132" s="2" t="s">
-        <v>464</v>
-      </c>
       <c r="E132" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="G132" s="12" t="s">
         <v>494</v>
       </c>
-      <c r="F132" s="2" t="s">
-        <v>476</v>
-      </c>
-      <c r="G132" s="12" t="s">
+      <c r="H132" s="13" t="s">
         <v>495</v>
-      </c>
-      <c r="H132" s="13" t="s">
-        <v>496</v>
       </c>
       <c r="I132" s="8" t="s">
         <v>20</v>
@@ -8605,10 +8563,10 @@
         <v>348</v>
       </c>
       <c r="K132" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="L132" s="6" t="s">
         <v>483</v>
-      </c>
-      <c r="L132" s="6" t="s">
-        <v>484</v>
       </c>
       <c r="M132" s="6" t="s">
         <v>24</v>
@@ -8619,25 +8577,25 @@
         <v>13</v>
       </c>
       <c r="B133" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C133" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="D133" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="D133" s="6" t="s">
-        <v>464</v>
-      </c>
       <c r="E133" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="F133" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="G133" s="14" t="s">
         <v>497</v>
       </c>
-      <c r="F133" s="6" t="s">
-        <v>480</v>
-      </c>
-      <c r="G133" s="14" t="s">
+      <c r="H133" s="13" t="s">
         <v>498</v>
-      </c>
-      <c r="H133" s="13" t="s">
-        <v>499</v>
       </c>
       <c r="I133" s="8" t="s">
         <v>20</v>
@@ -8646,10 +8604,10 @@
         <v>348</v>
       </c>
       <c r="K133" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="L133" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="L133" s="2" t="s">
-        <v>484</v>
       </c>
       <c r="M133" s="2" t="s">
         <v>24</v>
@@ -8660,25 +8618,25 @@
         <v>13</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C134" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D134" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D134" s="2" t="s">
-        <v>464</v>
-      </c>
       <c r="E134" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="G134" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="F134" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="G134" s="2" t="s">
+      <c r="H134" s="13" t="s">
         <v>501</v>
-      </c>
-      <c r="H134" s="13" t="s">
-        <v>502</v>
       </c>
       <c r="I134" s="8" t="s">
         <v>20</v>
@@ -8687,10 +8645,10 @@
         <v>337</v>
       </c>
       <c r="K134" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="L134" s="6" t="s">
         <v>483</v>
-      </c>
-      <c r="L134" s="6" t="s">
-        <v>484</v>
       </c>
       <c r="M134" s="6" t="s">
         <v>24</v>
@@ -8701,25 +8659,25 @@
         <v>13</v>
       </c>
       <c r="B135" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C135" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="D135" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="D135" s="6" t="s">
-        <v>464</v>
-      </c>
       <c r="E135" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="F135" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="G135" s="6" t="s">
         <v>503</v>
       </c>
-      <c r="F135" s="6" t="s">
-        <v>470</v>
-      </c>
-      <c r="G135" s="6" t="s">
+      <c r="H135" s="13" t="s">
         <v>504</v>
-      </c>
-      <c r="H135" s="13" t="s">
-        <v>505</v>
       </c>
       <c r="I135" s="8" t="s">
         <v>20</v>
@@ -8728,7 +8686,7 @@
         <v>348</v>
       </c>
       <c r="K135" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L135" s="2" t="s">
         <v>23</v>
@@ -8742,23 +8700,23 @@
         <v>13</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C136" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D136" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D136" s="2" t="s">
-        <v>464</v>
-      </c>
       <c r="E136" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="G136" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="F136" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="G136" s="2" t="s">
-        <v>508</v>
-      </c>
       <c r="H136" s="7" t="s">
         <v>57</v>
       </c>
@@ -8769,7 +8727,7 @@
         <v>57</v>
       </c>
       <c r="K136" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L136" s="6" t="s">
         <v>23</v>
@@ -8783,25 +8741,25 @@
         <v>13</v>
       </c>
       <c r="B137" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C137" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="D137" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="D137" s="6" t="s">
-        <v>464</v>
-      </c>
       <c r="E137" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="F137" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="G137" s="14" t="s">
         <v>509</v>
       </c>
-      <c r="F137" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G137" s="14" t="s">
+      <c r="H137" s="13" t="s">
         <v>510</v>
-      </c>
-      <c r="H137" s="13" t="s">
-        <v>511</v>
       </c>
       <c r="I137" s="8" t="s">
         <v>20</v>
@@ -8810,7 +8768,7 @@
         <v>348</v>
       </c>
       <c r="K137" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L137" s="2" t="s">
         <v>23</v>
@@ -8824,25 +8782,25 @@
         <v>13</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C138" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D138" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D138" s="2" t="s">
-        <v>464</v>
-      </c>
       <c r="E138" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="G138" s="12" t="s">
         <v>512</v>
       </c>
-      <c r="F138" s="2" t="s">
-        <v>480</v>
-      </c>
-      <c r="G138" s="12" t="s">
+      <c r="H138" s="13" t="s">
         <v>513</v>
-      </c>
-      <c r="H138" s="13" t="s">
-        <v>514</v>
       </c>
       <c r="I138" s="8" t="s">
         <v>20</v>
@@ -8851,7 +8809,7 @@
         <v>348</v>
       </c>
       <c r="K138" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L138" s="6" t="s">
         <v>23</v>
@@ -8865,22 +8823,22 @@
         <v>14</v>
       </c>
       <c r="B139" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="C139" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="C139" s="6" t="s">
+      <c r="D139" s="6" t="s">
         <v>516</v>
       </c>
-      <c r="D139" s="6" t="s">
+      <c r="E139" s="6" t="s">
         <v>517</v>
-      </c>
-      <c r="E139" s="6" t="s">
-        <v>518</v>
       </c>
       <c r="F139" s="6" t="s">
         <v>152</v>
       </c>
       <c r="G139" s="6" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="H139" s="7" t="s">
         <v>57</v>
@@ -8892,7 +8850,7 @@
         <v>57</v>
       </c>
       <c r="K139" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="L139" s="2" t="s">
         <v>23</v>
@@ -8906,34 +8864,34 @@
         <v>14</v>
       </c>
       <c r="B140" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="C140" s="2" t="s">
         <v>515</v>
       </c>
-      <c r="C140" s="2" t="s">
+      <c r="D140" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="D140" s="2" t="s">
-        <v>517</v>
-      </c>
       <c r="E140" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="F140" s="2" t="s">
         <v>156</v>
       </c>
       <c r="G140" s="12" t="s">
+        <v>520</v>
+      </c>
+      <c r="H140" s="13" t="s">
         <v>521</v>
       </c>
-      <c r="H140" s="13" t="s">
+      <c r="I140" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J140" s="14" t="s">
         <v>522</v>
       </c>
-      <c r="I140" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J140" s="14" t="s">
-        <v>523</v>
-      </c>
       <c r="K140" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L140" s="6" t="s">
         <v>23</v>
@@ -8947,25 +8905,25 @@
         <v>14</v>
       </c>
       <c r="B141" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="C141" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="C141" s="6" t="s">
+      <c r="D141" s="6" t="s">
         <v>516</v>
       </c>
-      <c r="D141" s="6" t="s">
-        <v>517</v>
-      </c>
       <c r="E141" s="6" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="F141" s="6" t="s">
         <v>161</v>
       </c>
       <c r="G141" s="14" t="s">
+        <v>524</v>
+      </c>
+      <c r="H141" s="18" t="s">
         <v>525</v>
-      </c>
-      <c r="H141" s="20" t="s">
-        <v>526</v>
       </c>
       <c r="I141" s="8" t="s">
         <v>20</v>
@@ -8974,7 +8932,7 @@
         <v>348</v>
       </c>
       <c r="K141" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L141" s="2" t="s">
         <v>23</v>
@@ -8988,22 +8946,22 @@
         <v>14</v>
       </c>
       <c r="B142" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="C142" s="2" t="s">
         <v>515</v>
       </c>
-      <c r="C142" s="2" t="s">
+      <c r="D142" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="D142" s="2" t="s">
-        <v>517</v>
-      </c>
       <c r="E142" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="F142" s="2" t="s">
         <v>183</v>
       </c>
       <c r="G142" s="12" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="H142" s="7" t="s">
         <v>57</v>
@@ -9015,7 +8973,7 @@
         <v>57</v>
       </c>
       <c r="K142" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L142" s="6" t="s">
         <v>23</v>
@@ -9029,25 +8987,25 @@
         <v>14</v>
       </c>
       <c r="B143" s="6" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C143" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="D143" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="D143" s="6" t="s">
+      <c r="E143" s="6" t="s">
         <v>530</v>
       </c>
-      <c r="E143" s="6" t="s">
+      <c r="F143" s="6" t="s">
         <v>531</v>
       </c>
-      <c r="F143" s="6" t="s">
+      <c r="G143" s="14" t="s">
         <v>532</v>
       </c>
-      <c r="G143" s="14" t="s">
+      <c r="H143" s="13" t="s">
         <v>533</v>
-      </c>
-      <c r="H143" s="13" t="s">
-        <v>534</v>
       </c>
       <c r="I143" s="8" t="s">
         <v>20</v>
@@ -9056,7 +9014,7 @@
         <v>348</v>
       </c>
       <c r="K143" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L143" s="2" t="s">
         <v>23</v>
@@ -9070,25 +9028,25 @@
         <v>14</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C144" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="D144" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="D144" s="2" t="s">
-        <v>530</v>
-      </c>
       <c r="E144" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="F144" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="F144" s="2" t="s">
+      <c r="G144" s="12" t="s">
         <v>536</v>
       </c>
-      <c r="G144" s="12" t="s">
+      <c r="H144" s="13" t="s">
         <v>537</v>
-      </c>
-      <c r="H144" s="13" t="s">
-        <v>538</v>
       </c>
       <c r="I144" s="8" t="s">
         <v>20</v>
@@ -9097,7 +9055,7 @@
         <v>348</v>
       </c>
       <c r="K144" s="6" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="L144" s="6" t="s">
         <v>23</v>
@@ -9111,23 +9069,23 @@
         <v>14</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C145" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="D145" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="D145" s="6" t="s">
-        <v>530</v>
-      </c>
       <c r="E145" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="F145" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="G145" s="14" t="s">
         <v>539</v>
       </c>
-      <c r="F145" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="G145" s="14" t="s">
-        <v>540</v>
-      </c>
       <c r="H145" s="7" t="s">
         <v>57</v>
       </c>
@@ -9138,7 +9096,7 @@
         <v>57</v>
       </c>
       <c r="K145" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L145" s="2" t="s">
         <v>23</v>
@@ -9152,25 +9110,25 @@
         <v>14</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C146" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="D146" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="D146" s="2" t="s">
-        <v>530</v>
-      </c>
       <c r="E146" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="F146" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="G146" s="12" t="s">
         <v>541</v>
       </c>
-      <c r="F146" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="G146" s="12" t="s">
+      <c r="H146" s="13" t="s">
         <v>542</v>
-      </c>
-      <c r="H146" s="13" t="s">
-        <v>543</v>
       </c>
       <c r="I146" s="8" t="s">
         <v>20</v>
@@ -9179,7 +9137,7 @@
         <v>348</v>
       </c>
       <c r="K146" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L146" s="6" t="s">
         <v>23</v>
@@ -9193,34 +9151,34 @@
         <v>14</v>
       </c>
       <c r="B147" s="6" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C147" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="D147" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="D147" s="6" t="s">
-        <v>530</v>
-      </c>
       <c r="E147" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="F147" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="G147" s="14" t="s">
         <v>544</v>
       </c>
-      <c r="F147" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="G147" s="14" t="s">
+      <c r="H147" s="13" t="s">
         <v>545</v>
       </c>
-      <c r="H147" s="13" t="s">
-        <v>546</v>
-      </c>
       <c r="I147" s="8" t="s">
         <v>20</v>
       </c>
       <c r="J147" s="12" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="K147" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L147" s="2" t="s">
         <v>23</v>
@@ -9234,25 +9192,25 @@
         <v>14</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C148" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="D148" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="D148" s="2" t="s">
-        <v>530</v>
-      </c>
       <c r="E148" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="F148" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="G148" s="12" t="s">
         <v>547</v>
       </c>
-      <c r="F148" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="G148" s="12" t="s">
+      <c r="H148" s="13" t="s">
         <v>548</v>
-      </c>
-      <c r="H148" s="13" t="s">
-        <v>549</v>
       </c>
       <c r="I148" s="8" t="s">
         <v>20</v>
@@ -9261,7 +9219,7 @@
         <v>348</v>
       </c>
       <c r="K148" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L148" s="6" t="s">
         <v>23</v>
@@ -9275,25 +9233,25 @@
         <v>14</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C149" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="D149" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="D149" s="6" t="s">
-        <v>530</v>
-      </c>
       <c r="E149" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="F149" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="G149" s="14" t="s">
         <v>550</v>
       </c>
-      <c r="F149" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="G149" s="14" t="s">
+      <c r="H149" s="13" t="s">
         <v>551</v>
-      </c>
-      <c r="H149" s="13" t="s">
-        <v>552</v>
       </c>
       <c r="I149" s="8" t="s">
         <v>20</v>
@@ -9302,7 +9260,7 @@
         <v>348</v>
       </c>
       <c r="K149" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="L149" s="2" t="s">
         <v>23</v>
@@ -9316,25 +9274,25 @@
         <v>14</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C150" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="D150" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="D150" s="2" t="s">
-        <v>530</v>
-      </c>
       <c r="E150" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="G150" s="12" t="s">
         <v>553</v>
       </c>
-      <c r="F150" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="G150" s="12" t="s">
+      <c r="H150" s="13" t="s">
         <v>554</v>
-      </c>
-      <c r="H150" s="13" t="s">
-        <v>555</v>
       </c>
       <c r="I150" s="8" t="s">
         <v>20</v>
@@ -9343,10 +9301,10 @@
         <v>348</v>
       </c>
       <c r="K150" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="L150" s="6" t="s">
         <v>556</v>
-      </c>
-      <c r="L150" s="6" t="s">
-        <v>557</v>
       </c>
       <c r="M150" s="6" t="s">
         <v>24</v>
@@ -9357,25 +9315,25 @@
         <v>14</v>
       </c>
       <c r="B151" s="6" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C151" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="D151" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="D151" s="6" t="s">
-        <v>530</v>
-      </c>
       <c r="E151" s="6" t="s">
+        <v>557</v>
+      </c>
+      <c r="F151" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="G151" s="14" t="s">
         <v>558</v>
       </c>
-      <c r="F151" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="G151" s="14" t="s">
+      <c r="H151" s="13" t="s">
         <v>559</v>
-      </c>
-      <c r="H151" s="13" t="s">
-        <v>560</v>
       </c>
       <c r="I151" s="8" t="s">
         <v>20</v>
@@ -9384,10 +9342,10 @@
         <v>348</v>
       </c>
       <c r="K151" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="L151" s="2" t="s">
         <v>556</v>
-      </c>
-      <c r="L151" s="2" t="s">
-        <v>557</v>
       </c>
       <c r="M151" s="2" t="s">
         <v>24</v>
@@ -9398,25 +9356,25 @@
         <v>14</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C152" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="D152" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="D152" s="2" t="s">
-        <v>530</v>
-      </c>
       <c r="E152" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="F152" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="G152" s="12" t="s">
         <v>561</v>
       </c>
-      <c r="F152" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="G152" s="12" t="s">
+      <c r="H152" s="13" t="s">
         <v>562</v>
-      </c>
-      <c r="H152" s="13" t="s">
-        <v>563</v>
       </c>
       <c r="I152" s="8" t="s">
         <v>20</v>
@@ -9425,10 +9383,10 @@
         <v>348</v>
       </c>
       <c r="K152" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="L152" s="6" t="s">
         <v>556</v>
-      </c>
-      <c r="L152" s="6" t="s">
-        <v>557</v>
       </c>
       <c r="M152" s="6" t="s">
         <v>24</v>
@@ -9439,25 +9397,25 @@
         <v>15</v>
       </c>
       <c r="B153" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="C153" s="6" t="s">
         <v>564</v>
       </c>
-      <c r="C153" s="6" t="s">
+      <c r="D153" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="D153" s="6" t="s">
+      <c r="E153" s="6" t="s">
         <v>566</v>
-      </c>
-      <c r="E153" s="6" t="s">
-        <v>567</v>
       </c>
       <c r="F153" s="6" t="s">
         <v>152</v>
       </c>
       <c r="G153" s="14" t="s">
+        <v>567</v>
+      </c>
+      <c r="H153" s="13" t="s">
         <v>568</v>
-      </c>
-      <c r="H153" s="13" t="s">
-        <v>569</v>
       </c>
       <c r="I153" s="8" t="s">
         <v>20</v>
@@ -9466,10 +9424,10 @@
         <v>348</v>
       </c>
       <c r="K153" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="L153" s="2" t="s">
         <v>556</v>
-      </c>
-      <c r="L153" s="2" t="s">
-        <v>557</v>
       </c>
       <c r="M153" s="2" t="s">
         <v>24</v>
@@ -9480,25 +9438,25 @@
         <v>15</v>
       </c>
       <c r="B154" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C154" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="C154" s="2" t="s">
+      <c r="D154" s="2" t="s">
         <v>565</v>
       </c>
-      <c r="D154" s="2" t="s">
-        <v>566</v>
-      </c>
       <c r="E154" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="F154" s="2" t="s">
         <v>156</v>
       </c>
       <c r="G154" s="12" t="s">
+        <v>570</v>
+      </c>
+      <c r="H154" s="13" t="s">
         <v>571</v>
-      </c>
-      <c r="H154" s="13" t="s">
-        <v>572</v>
       </c>
       <c r="I154" s="8" t="s">
         <v>20</v>
@@ -9507,7 +9465,7 @@
         <v>348</v>
       </c>
       <c r="K154" s="6" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="L154" s="6" t="s">
         <v>23</v>
@@ -9521,25 +9479,25 @@
         <v>15</v>
       </c>
       <c r="B155" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="C155" s="6" t="s">
         <v>564</v>
       </c>
-      <c r="C155" s="6" t="s">
+      <c r="D155" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="D155" s="6" t="s">
-        <v>566</v>
-      </c>
       <c r="E155" s="6" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="F155" s="6" t="s">
         <v>161</v>
       </c>
       <c r="G155" s="14" t="s">
+        <v>574</v>
+      </c>
+      <c r="H155" s="13" t="s">
         <v>575</v>
-      </c>
-      <c r="H155" s="13" t="s">
-        <v>576</v>
       </c>
       <c r="I155" s="8" t="s">
         <v>20</v>
@@ -9548,7 +9506,7 @@
         <v>348</v>
       </c>
       <c r="K155" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="L155" s="2" t="s">
         <v>23</v>
@@ -9562,22 +9520,22 @@
         <v>15</v>
       </c>
       <c r="B156" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C156" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="C156" s="2" t="s">
+      <c r="D156" s="2" t="s">
         <v>565</v>
       </c>
-      <c r="D156" s="2" t="s">
-        <v>566</v>
-      </c>
       <c r="E156" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="F156" s="2" t="s">
         <v>183</v>
       </c>
       <c r="G156" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="H156" s="7" t="s">
         <v>57</v>
@@ -9589,7 +9547,7 @@
         <v>57</v>
       </c>
       <c r="K156" s="6" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="L156" s="6" t="s">
         <v>23</v>
@@ -9603,19 +9561,19 @@
         <v>15</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C157" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="D157" s="2" t="s">
         <v>579</v>
       </c>
-      <c r="D157" s="2" t="s">
+      <c r="E157" s="2" t="s">
         <v>580</v>
       </c>
-      <c r="E157" s="2" t="s">
+      <c r="F157" s="2" t="s">
         <v>581</v>
-      </c>
-      <c r="F157" s="2" t="s">
-        <v>582</v>
       </c>
       <c r="G157" s="2" t="s">
         <v>229</v>
@@ -9626,10 +9584,10 @@
       </c>
       <c r="J157" s="14"/>
       <c r="K157" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="L157" s="6" t="s">
         <v>583</v>
-      </c>
-      <c r="L157" s="6" t="s">
-        <v>584</v>
       </c>
       <c r="M157" s="6" t="s">
         <v>24</v>
@@ -9640,25 +9598,25 @@
         <v>15</v>
       </c>
       <c r="B158" s="6" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C158" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D158" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="D158" s="6" t="s">
-        <v>580</v>
-      </c>
       <c r="E158" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="F158" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="G158" s="14" t="s">
         <v>585</v>
       </c>
-      <c r="F158" s="6" t="s">
-        <v>582</v>
-      </c>
-      <c r="G158" s="14" t="s">
+      <c r="H158" s="13" t="s">
         <v>586</v>
-      </c>
-      <c r="H158" s="13" t="s">
-        <v>587</v>
       </c>
       <c r="I158" s="8" t="s">
         <v>20</v>
@@ -9667,10 +9625,10 @@
         <v>348</v>
       </c>
       <c r="K158" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="L158" s="2" t="s">
         <v>583</v>
-      </c>
-      <c r="L158" s="2" t="s">
-        <v>584</v>
       </c>
       <c r="M158" s="2" t="s">
         <v>24</v>
@@ -9681,37 +9639,37 @@
         <v>15</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C159" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="D159" s="2" t="s">
         <v>579</v>
       </c>
-      <c r="D159" s="2" t="s">
-        <v>580</v>
-      </c>
       <c r="E159" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="G159" s="2" t="s">
         <v>588</v>
       </c>
-      <c r="F159" s="2" t="s">
+      <c r="H159" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I159" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J159" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K159" s="6" t="s">
         <v>582</v>
       </c>
-      <c r="G159" s="2" t="s">
-        <v>589</v>
-      </c>
-      <c r="H159" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="I159" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J159" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="K159" s="6" t="s">
+      <c r="L159" s="6" t="s">
         <v>583</v>
-      </c>
-      <c r="L159" s="6" t="s">
-        <v>584</v>
       </c>
       <c r="M159" s="6" t="s">
         <v>24</v>
@@ -9722,25 +9680,25 @@
         <v>15</v>
       </c>
       <c r="B160" s="6" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C160" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D160" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="D160" s="6" t="s">
-        <v>580</v>
-      </c>
       <c r="E160" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="F160" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="G160" s="14" t="s">
         <v>590</v>
       </c>
-      <c r="F160" s="6" t="s">
-        <v>582</v>
-      </c>
-      <c r="G160" s="14" t="s">
+      <c r="H160" s="13" t="s">
         <v>591</v>
-      </c>
-      <c r="H160" s="13" t="s">
-        <v>592</v>
       </c>
       <c r="I160" s="8" t="s">
         <v>20</v>
@@ -9749,10 +9707,10 @@
         <v>348</v>
       </c>
       <c r="K160" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="L160" s="2" t="s">
         <v>583</v>
-      </c>
-      <c r="L160" s="2" t="s">
-        <v>584</v>
       </c>
       <c r="M160" s="2" t="s">
         <v>24</v>
@@ -9763,25 +9721,25 @@
         <v>16</v>
       </c>
       <c r="B161" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="C161" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="C161" s="2" t="s">
+      <c r="D161" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="D161" s="2" t="s">
+      <c r="E161" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="E161" s="2" t="s">
+      <c r="F161" s="2" t="s">
         <v>596</v>
       </c>
-      <c r="F161" s="2" t="s">
+      <c r="G161" s="12" t="s">
         <v>597</v>
       </c>
-      <c r="G161" s="12" t="s">
+      <c r="H161" s="13" t="s">
         <v>598</v>
-      </c>
-      <c r="H161" s="13" t="s">
-        <v>599</v>
       </c>
       <c r="I161" s="8" t="s">
         <v>20</v>
@@ -9790,10 +9748,10 @@
         <v>348</v>
       </c>
       <c r="K161" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="L161" s="6" t="s">
         <v>583</v>
-      </c>
-      <c r="L161" s="6" t="s">
-        <v>584</v>
       </c>
       <c r="M161" s="6" t="s">
         <v>24</v>
@@ -9804,19 +9762,19 @@
         <v>16</v>
       </c>
       <c r="B162" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="C162" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="C162" s="6" t="s">
+      <c r="D162" s="6" t="s">
         <v>594</v>
       </c>
-      <c r="D162" s="6" t="s">
-        <v>595</v>
-      </c>
       <c r="E162" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="F162" s="6" t="s">
         <v>600</v>
-      </c>
-      <c r="F162" s="6" t="s">
-        <v>601</v>
       </c>
       <c r="G162" s="6" t="s">
         <v>213</v>
@@ -9831,10 +9789,10 @@
         <v>57</v>
       </c>
       <c r="K162" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="L162" s="2" t="s">
         <v>583</v>
-      </c>
-      <c r="L162" s="2" t="s">
-        <v>584</v>
       </c>
       <c r="M162" s="2" t="s">
         <v>24</v>
@@ -9845,23 +9803,23 @@
         <v>16</v>
       </c>
       <c r="B163" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="C163" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="C163" s="2" t="s">
+      <c r="D163" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="D163" s="2" t="s">
-        <v>595</v>
-      </c>
       <c r="E163" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="F163" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="G163" s="2" t="s">
         <v>602</v>
       </c>
-      <c r="F163" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="G163" s="2" t="s">
-        <v>603</v>
-      </c>
       <c r="H163" s="7" t="s">
         <v>57</v>
       </c>
@@ -9872,10 +9830,10 @@
         <v>57</v>
       </c>
       <c r="K163" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="L163" s="6" t="s">
         <v>583</v>
-      </c>
-      <c r="L163" s="6" t="s">
-        <v>584</v>
       </c>
       <c r="M163" s="6" t="s">
         <v>24</v>
@@ -9886,23 +9844,23 @@
         <v>16</v>
       </c>
       <c r="B164" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="C164" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="C164" s="6" t="s">
+      <c r="D164" s="6" t="s">
         <v>594</v>
       </c>
-      <c r="D164" s="6" t="s">
-        <v>595</v>
-      </c>
       <c r="E164" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="F164" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="G164" s="6" t="s">
         <v>604</v>
       </c>
-      <c r="F164" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="G164" s="6" t="s">
-        <v>605</v>
-      </c>
       <c r="H164" s="7" t="s">
         <v>57</v>
       </c>
@@ -9913,10 +9871,10 @@
         <v>57</v>
       </c>
       <c r="K164" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="L164" s="2" t="s">
         <v>583</v>
-      </c>
-      <c r="L164" s="2" t="s">
-        <v>584</v>
       </c>
       <c r="M164" s="2" t="s">
         <v>24</v>
@@ -9927,23 +9885,23 @@
         <v>16</v>
       </c>
       <c r="B165" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="C165" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="C165" s="2" t="s">
+      <c r="D165" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="D165" s="2" t="s">
-        <v>595</v>
-      </c>
       <c r="E165" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="F165" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="F165" s="2" t="s">
+      <c r="G165" s="2" t="s">
         <v>607</v>
       </c>
-      <c r="G165" s="2" t="s">
-        <v>608</v>
-      </c>
       <c r="H165" s="7" t="s">
         <v>57</v>
       </c>
@@ -9954,10 +9912,10 @@
         <v>57</v>
       </c>
       <c r="K165" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="L165" s="6" t="s">
         <v>583</v>
-      </c>
-      <c r="L165" s="6" t="s">
-        <v>584</v>
       </c>
       <c r="M165" s="6" t="s">
         <v>24</v>
@@ -9968,22 +9926,22 @@
         <v>16</v>
       </c>
       <c r="B166" s="6" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C166" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="D166" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="E166" s="6" t="s">
         <v>609</v>
       </c>
-      <c r="D166" s="6" t="s">
-        <v>595</v>
-      </c>
-      <c r="E166" s="6" t="s">
+      <c r="F166" s="6" t="s">
         <v>610</v>
       </c>
-      <c r="F166" s="6" t="s">
+      <c r="G166" s="6" t="s">
         <v>611</v>
-      </c>
-      <c r="G166" s="6" t="s">
-        <v>612</v>
       </c>
       <c r="H166" s="13" t="s">
         <v>229</v>
@@ -9995,10 +9953,10 @@
         <v>348</v>
       </c>
       <c r="K166" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L166" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M166" s="2" t="s">
         <v>24</v>
@@ -10009,25 +9967,25 @@
         <v>16</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E167" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="F167" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="G167" s="12" t="s">
         <v>614</v>
       </c>
-      <c r="F167" s="2" t="s">
-        <v>611</v>
-      </c>
-      <c r="G167" s="12" t="s">
+      <c r="H167" s="13" t="s">
         <v>615</v>
-      </c>
-      <c r="H167" s="13" t="s">
-        <v>616</v>
       </c>
       <c r="I167" s="8" t="s">
         <v>20</v>
@@ -10036,10 +9994,10 @@
         <v>348</v>
       </c>
       <c r="K167" s="6" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L167" s="6" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M167" s="6" t="s">
         <v>24</v>
@@ -10050,22 +10008,22 @@
         <v>16</v>
       </c>
       <c r="B168" s="6" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C168" s="6" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D168" s="6" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E168" s="6" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="F168" s="6" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="G168" s="6" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="H168" s="7" t="s">
         <v>57</v>
@@ -10077,10 +10035,10 @@
         <v>57</v>
       </c>
       <c r="K168" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L168" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M168" s="2" t="s">
         <v>24</v>
@@ -10091,25 +10049,25 @@
         <v>16</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E169" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="F169" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="G169" s="2" t="s">
         <v>618</v>
       </c>
-      <c r="F169" s="2" t="s">
-        <v>611</v>
-      </c>
-      <c r="G169" s="2" t="s">
+      <c r="H169" s="13" t="s">
         <v>619</v>
-      </c>
-      <c r="H169" s="13" t="s">
-        <v>620</v>
       </c>
       <c r="I169" s="8" t="s">
         <v>20</v>
@@ -10118,10 +10076,10 @@
         <v>348</v>
       </c>
       <c r="K169" s="6" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L169" s="6" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M169" s="6" t="s">
         <v>24</v>
@@ -10132,37 +10090,37 @@
         <v>16</v>
       </c>
       <c r="B170" s="6" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C170" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="D170" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="E170" s="6" t="s">
         <v>621</v>
       </c>
-      <c r="D170" s="6" t="s">
-        <v>595</v>
-      </c>
-      <c r="E170" s="6" t="s">
+      <c r="F170" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="G170" s="6" t="s">
         <v>622</v>
       </c>
-      <c r="F170" s="6" t="s">
-        <v>611</v>
-      </c>
-      <c r="G170" s="6" t="s">
+      <c r="H170" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I170" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J170" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K170" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="H170" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="I170" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J170" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="K170" s="2" t="s">
+      <c r="L170" s="2" t="s">
         <v>624</v>
-      </c>
-      <c r="L170" s="2" t="s">
-        <v>625</v>
       </c>
       <c r="M170" s="2" t="s">
         <v>24</v>
@@ -10173,19 +10131,19 @@
         <v>16</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="F171" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="G171" s="2" t="s">
         <v>293</v>
@@ -10200,10 +10158,10 @@
         <v>57</v>
       </c>
       <c r="K171" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="L171" s="6" t="s">
         <v>624</v>
-      </c>
-      <c r="L171" s="6" t="s">
-        <v>625</v>
       </c>
       <c r="M171" s="6" t="s">
         <v>24</v>
@@ -10214,19 +10172,19 @@
         <v>16</v>
       </c>
       <c r="B172" s="6" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C172" s="6" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D172" s="6" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E172" s="6" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F172" s="6" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="G172" s="6" t="s">
         <v>340</v>
@@ -10241,10 +10199,10 @@
         <v>57</v>
       </c>
       <c r="K172" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="L172" s="2" t="s">
         <v>624</v>
-      </c>
-      <c r="L172" s="2" t="s">
-        <v>625</v>
       </c>
       <c r="M172" s="2" t="s">
         <v>24</v>
@@ -10255,22 +10213,22 @@
         <v>16</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E173" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F173" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="G173" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="H173" s="7" t="s">
         <v>57</v>
@@ -10282,10 +10240,10 @@
         <v>57</v>
       </c>
       <c r="K173" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="L173" s="6" t="s">
         <v>624</v>
-      </c>
-      <c r="L173" s="6" t="s">
-        <v>625</v>
       </c>
       <c r="M173" s="6" t="s">
         <v>24</v>
@@ -10296,23 +10254,23 @@
         <v>16</v>
       </c>
       <c r="B174" s="6" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C174" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="D174" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="E174" s="6" t="s">
         <v>629</v>
       </c>
-      <c r="D174" s="6" t="s">
-        <v>595</v>
-      </c>
-      <c r="E174" s="6" t="s">
+      <c r="F174" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="F174" s="6" t="s">
+      <c r="G174" s="6" t="s">
         <v>631</v>
       </c>
-      <c r="G174" s="6" t="s">
-        <v>632</v>
-      </c>
       <c r="H174" s="7" t="s">
         <v>57</v>
       </c>
@@ -10323,10 +10281,10 @@
         <v>57</v>
       </c>
       <c r="K174" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="L174" s="2" t="s">
         <v>624</v>
-      </c>
-      <c r="L174" s="2" t="s">
-        <v>625</v>
       </c>
       <c r="M174" s="2" t="s">
         <v>24</v>
@@ -10337,23 +10295,23 @@
         <v>16</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E175" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="F175" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="G175" s="2" t="s">
         <v>633</v>
       </c>
-      <c r="F175" s="2" t="s">
-        <v>631</v>
-      </c>
-      <c r="G175" s="2" t="s">
-        <v>634</v>
-      </c>
       <c r="H175" s="7" t="s">
         <v>57</v>
       </c>
@@ -10364,10 +10322,10 @@
         <v>57</v>
       </c>
       <c r="K175" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="L175" s="6" t="s">
         <v>624</v>
-      </c>
-      <c r="L175" s="6" t="s">
-        <v>625</v>
       </c>
       <c r="M175" s="6" t="s">
         <v>24</v>
@@ -10384,7 +10342,7 @@
         <v>57</v>
       </c>
       <c r="K176" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="L176" s="6" t="s">
         <v>23</v>
@@ -10404,7 +10362,7 @@
         <v>57</v>
       </c>
       <c r="K177" s="2" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="L177" s="2" t="s">
         <v>23</v>
@@ -10424,7 +10382,7 @@
         <v>57</v>
       </c>
       <c r="K178" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="L178" s="6" t="s">
         <v>23</v>
@@ -10444,7 +10402,7 @@
         <v>57</v>
       </c>
       <c r="K179" s="2" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="L179" s="2" t="s">
         <v>23</v>
@@ -10464,7 +10422,7 @@
         <v>57</v>
       </c>
       <c r="K180" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="L180" s="6" t="s">
         <v>23</v>
@@ -10484,7 +10442,7 @@
         <v>57</v>
       </c>
       <c r="K181" s="2" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="L181" s="2" t="s">
         <v>23</v>
@@ -10504,7 +10462,7 @@
         <v>57</v>
       </c>
       <c r="K182" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="L182" s="6" t="s">
         <v>23</v>
@@ -10524,7 +10482,7 @@
         <v>57</v>
       </c>
       <c r="K183" s="2" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="L183" s="2" t="s">
         <v>23</v>
@@ -10544,10 +10502,10 @@
         <v>57</v>
       </c>
       <c r="K184" s="6" t="s">
+        <v>636</v>
+      </c>
+      <c r="L184" s="6" t="s">
         <v>637</v>
-      </c>
-      <c r="L184" s="6" t="s">
-        <v>638</v>
       </c>
       <c r="M184" s="6" t="s">
         <v>24</v>
@@ -10564,10 +10522,10 @@
         <v>57</v>
       </c>
       <c r="K185" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="L185" s="2" t="s">
         <v>637</v>
-      </c>
-      <c r="L185" s="2" t="s">
-        <v>638</v>
       </c>
       <c r="M185" s="2" t="s">
         <v>24</v>
@@ -10584,10 +10542,10 @@
         <v>57</v>
       </c>
       <c r="K186" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="L186" s="2" t="s">
         <v>637</v>
-      </c>
-      <c r="L186" s="2" t="s">
-        <v>638</v>
       </c>
       <c r="M186" s="2" t="s">
         <v>24</v>
@@ -10625,66 +10583,66 @@
   <sheetData>
     <row r="1" ht="33.9" customHeight="1" spans="1:2">
       <c r="A1" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>639</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>640</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
+        <v>640</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>641</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>642</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>643</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>644</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>645</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>646</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>647</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>648</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>649</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>650</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>651</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>652</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>653</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>654</v>
       </c>
     </row>
   </sheetData>
@@ -10708,7 +10666,7 @@
   <sheetData>
     <row r="1" ht="33.9" customHeight="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -10717,10 +10675,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>655</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>656</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:5">
@@ -10745,16 +10703,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>658</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>659</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>660</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:5">
@@ -10762,16 +10720,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>662</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>663</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:5">
@@ -10779,13 +10737,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>23</v>
@@ -10881,13 +10839,13 @@
         <v>5</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>665</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>666</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>667</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>23</v>
@@ -10898,13 +10856,13 @@
         <v>6</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>668</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>669</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>670</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>23</v>
@@ -11136,13 +11094,13 @@
         <v>13</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>463</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>464</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>23</v>
@@ -11153,16 +11111,16 @@
         <v>13</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>440</v>
-      </c>
       <c r="E27" s="2" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1" spans="1:5">
@@ -11170,16 +11128,16 @@
         <v>14</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>515</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>517</v>
-      </c>
       <c r="E28" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1" spans="1:5">
@@ -11187,13 +11145,13 @@
         <v>14</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>529</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>530</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>23</v>
@@ -11204,16 +11162,16 @@
         <v>15</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>565</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>566</v>
-      </c>
       <c r="E30" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1" spans="1:5">
@@ -11221,16 +11179,16 @@
         <v>15</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>579</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>580</v>
-      </c>
       <c r="E31" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1" spans="1:5">
@@ -11238,16 +11196,16 @@
         <v>16</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>595</v>
-      </c>
       <c r="E32" s="2" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="33" ht="48" customHeight="1" spans="1:5">
@@ -11255,13 +11213,13 @@
         <v>16</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>23</v>
@@ -11272,13 +11230,13 @@
         <v>16</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>23</v>
@@ -11289,13 +11247,13 @@
         <v>16</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>23</v>
@@ -11306,16 +11264,16 @@
         <v>17</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>671</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>672</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>673</v>
-      </c>
       <c r="E36" s="2" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
   </sheetData>

</xml_diff>